<commit_message>
SALVAMED para el Sanatorio El Roble: despacho a servicios en vez de ventas
- La farmacia interna despacha a servicios (Emergencia, Encamamiento, Cuidados
  Intensivos, Sala de operaciones, Traumatología, Ambulancia), sin datos de
  pacientes ni cobros. La lista sale de lo que publica el sanatorio y se edita
  en Configuración.
- El panel de dinero pasa a costos: costo de lo consumido total y por servicio,
  compras recibidas y comprometidas. Se quita el precio de venta.
- Operación de 24 horas todos los días (fuentes: TuSalud y Facebook).
- Simulación del sanatorio: cada servicio pide con su propio horario y su propia
  secuencia aleatoria; aviso de aumento como evento; escenario de aumento desde
  el día 15.
- El módulo de tareas de fondo se renombra a app/tareas.py.
- README, modelo y guion actualizados con datos verificados de la semilla 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/ejemplo_simulado.xlsx
+++ b/datos/ejemplo_simulado.xlsx
@@ -475,7 +475,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Historial diario: ventas de días completos (una fila por día y medicamento). No mueve existencias: solo alimenta μD y σD.</t>
+          <t xml:space="preserve">  Historial diario: unidades despachadas a los servicios en días completos (una fila por día y medicamento). No mueve existencias: solo alimenta μD y σD.</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Un día observado sin ventas se escribe con cantidad 0; un día sin registro simplemente no se escribe.</t>
+          <t>Un día observado sin despachos se escribe con cantidad 0; un día sin registro simplemente no se escribe.</t>
         </is>
       </c>
     </row>
@@ -523,14 +523,14 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TODO ES SIMULADO: catálogo, costos, precios y existencias inventados; 45 días de ventas GENERADOS con la semilla 2026.</t>
+          <t>TODO ES SIMULADO: catálogo, costos y existencias inventados; 45 días de consumo GENERADOS con la semilla 2026.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Solo los nombres de los medicamentos están contextualizados en El Roble. No son datos entregados por El Roble.</t>
+          <t>Solo los nombres de los medicamentos están contextualizados en el Sanatorio El Roble. No son datos entregados por el sanatorio.</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -562,11 +562,10 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -607,25 +606,20 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>precio_venta_q</t>
+          <t>unidades_paquete</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>unidades_paquete</t>
+          <t>existencia</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>existencia</t>
+          <t>tiempo_entrega_dias</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>tiempo_entrega_dias</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>vencimiento_proximo</t>
         </is>
@@ -665,16 +659,13 @@
       <c r="G2" s="4" t="n">
         <v>12.5</v>
       </c>
-      <c r="H2" s="4" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="H2" t="n">
         <v>10</v>
       </c>
+      <c r="I2" s="4" t="n">
+        <v>60</v>
+      </c>
       <c r="J2" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="K2" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -712,16 +703,13 @@
       <c r="G3" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="H3" s="4" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="I3" t="n">
+      <c r="H3" t="n">
         <v>12</v>
       </c>
+      <c r="I3" s="4" t="n">
+        <v>150</v>
+      </c>
       <c r="J3" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="K3" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -759,16 +747,13 @@
       <c r="G4" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="H4" s="4" t="n">
-        <v>7.45</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="H4" t="n">
         <v>20</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>300</v>
+      </c>
       <c r="J4" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="K4" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -806,16 +791,13 @@
       <c r="G5" s="4" t="n">
         <v>5.9</v>
       </c>
-      <c r="H5" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="H5" t="n">
         <v>10</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>90</v>
+      </c>
       <c r="J5" s="4" t="n">
-        <v>90</v>
-      </c>
-      <c r="K5" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -853,16 +835,13 @@
       <c r="G6" s="4" t="n">
         <v>4.7</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>6.35</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
         <v>10</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="J6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="K6" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -900,16 +879,13 @@
       <c r="G7" s="4" t="n">
         <v>4.1</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="I7" t="n">
+      <c r="H7" t="n">
         <v>20</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>120</v>
+      </c>
       <c r="J7" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="K7" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -947,16 +923,13 @@
       <c r="G8" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="H8" s="4" t="n">
-        <v>118.8</v>
-      </c>
-      <c r="I8" t="n">
+      <c r="H8" t="n">
         <v>1</v>
       </c>
+      <c r="I8" s="4" t="n">
+        <v>14</v>
+      </c>
       <c r="J8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="K8" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -994,16 +967,13 @@
       <c r="G9" s="4" t="n">
         <v>7.5</v>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="H9" t="n">
         <v>10</v>
       </c>
+      <c r="I9" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="J9" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="K9" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1066,7 +1036,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1086,7 +1056,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -1106,7 +1076,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -1126,7 +1096,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -1146,7 +1116,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -1166,7 +1136,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -1186,7 +1156,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1206,7 +1176,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1226,7 +1196,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1246,7 +1216,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1586,7 +1556,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29">
@@ -1606,7 +1576,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -1626,7 +1596,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
@@ -1646,7 +1616,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32">
@@ -1686,7 +1656,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1706,7 +1676,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -1726,7 +1696,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36">
@@ -1746,7 +1716,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37">
@@ -1766,7 +1736,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -1786,7 +1756,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
@@ -1826,7 +1796,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1846,7 +1816,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1866,7 +1836,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43">
@@ -1886,7 +1856,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44">
@@ -1926,7 +1896,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
@@ -1966,7 +1936,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48">
@@ -1986,7 +1956,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -2006,7 +1976,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -2026,7 +1996,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51">
@@ -2046,7 +2016,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52">
@@ -2066,7 +2036,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="53">
@@ -2086,7 +2056,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54">
@@ -2106,7 +2076,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -2126,7 +2096,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56">
@@ -2146,7 +2116,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -2166,7 +2136,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -2186,7 +2156,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -2206,7 +2176,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60">
@@ -2226,7 +2196,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61">
@@ -2246,7 +2216,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62">
@@ -2266,7 +2236,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63">
@@ -2286,7 +2256,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64">
@@ -2306,7 +2276,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -2326,7 +2296,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -2346,7 +2316,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67">
@@ -2366,7 +2336,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68">
@@ -2386,7 +2356,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="69">
@@ -2406,7 +2376,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="70">
@@ -2426,7 +2396,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71">
@@ -2446,7 +2416,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72">
@@ -2466,7 +2436,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -2486,7 +2456,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
@@ -2546,7 +2516,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="77">
@@ -2566,7 +2536,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78">
@@ -2586,7 +2556,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
@@ -2606,7 +2576,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
@@ -2646,7 +2616,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -2666,7 +2636,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -2686,7 +2656,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="84">
@@ -2706,7 +2676,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="85">
@@ -2726,7 +2696,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
@@ -2766,7 +2736,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88">
@@ -2826,7 +2796,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91">
@@ -2846,7 +2816,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="92">
@@ -2866,7 +2836,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="93">
@@ -2886,7 +2856,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="94">
@@ -2906,7 +2876,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
@@ -2926,7 +2896,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96">
@@ -2946,7 +2916,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -2986,7 +2956,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="99">
@@ -3006,7 +2976,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="100">
@@ -3026,7 +2996,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="101">
@@ -3046,7 +3016,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102">
@@ -3066,7 +3036,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="103">
@@ -3086,7 +3056,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104">
@@ -3106,7 +3076,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
@@ -3126,7 +3096,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -3146,7 +3116,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="107">
@@ -3166,7 +3136,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="108">
@@ -3186,7 +3156,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="109">
@@ -3206,7 +3176,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="110">
@@ -3226,7 +3196,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111">
@@ -3246,7 +3216,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="112">
@@ -3266,7 +3236,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -3286,7 +3256,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -3306,7 +3276,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="115">
@@ -3326,7 +3296,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="116">
@@ -3346,7 +3316,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="117">
@@ -3366,7 +3336,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118">
@@ -3386,7 +3356,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119">
@@ -3426,7 +3396,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
@@ -3446,7 +3416,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -3466,7 +3436,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="123">
@@ -3486,7 +3456,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="124">
@@ -3506,7 +3476,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="125">
@@ -3526,7 +3496,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="126">
@@ -3546,7 +3516,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="127">
@@ -3566,7 +3536,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
@@ -3586,7 +3556,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129">
@@ -3606,7 +3576,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -3626,7 +3596,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131">
@@ -3646,7 +3616,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="132">
@@ -3666,7 +3636,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="133">
@@ -3686,7 +3656,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="134">
@@ -3706,7 +3676,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135">
@@ -3726,7 +3696,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="136">
@@ -3746,7 +3716,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="137">
@@ -3766,7 +3736,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
@@ -3786,7 +3756,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
@@ -3806,7 +3776,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="140">
@@ -3826,7 +3796,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="141">
@@ -3846,7 +3816,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="142">
@@ -3886,7 +3856,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="144">
@@ -3906,7 +3876,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -3946,7 +3916,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147">
@@ -3966,7 +3936,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="148">
@@ -3986,7 +3956,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
     </row>
     <row r="149">
@@ -4006,7 +3976,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150">
@@ -4026,7 +3996,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="151">
@@ -4046,7 +4016,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="152">
@@ -4066,7 +4036,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -4086,7 +4056,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154">
@@ -4106,7 +4076,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155">
@@ -4126,7 +4096,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="156">
@@ -4146,7 +4116,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="157">
@@ -4186,7 +4156,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="159">
@@ -4226,7 +4196,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -4246,7 +4216,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -4286,7 +4256,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="164">
@@ -4306,7 +4276,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="165">
@@ -4326,7 +4296,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="166">
@@ -4346,7 +4316,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167">
@@ -4366,7 +4336,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="168">
@@ -4386,7 +4356,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -4426,7 +4396,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="171">
@@ -4446,7 +4416,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="172">
@@ -4466,7 +4436,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="173">
@@ -4486,7 +4456,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="174">
@@ -4506,7 +4476,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -4526,7 +4496,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176">
@@ -4546,7 +4516,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
@@ -4566,7 +4536,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
@@ -4586,7 +4556,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="179">
@@ -4606,7 +4576,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="180">
@@ -4626,7 +4596,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="181">
@@ -4646,7 +4616,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="182">
@@ -4666,7 +4636,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="183">
@@ -4686,7 +4656,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="184">
@@ -4726,7 +4696,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="186">
@@ -4746,7 +4716,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="187">
@@ -4766,7 +4736,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188">
@@ -4786,7 +4756,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="189">
@@ -4806,7 +4776,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="190">
@@ -4826,7 +4796,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="191">
@@ -4846,7 +4816,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="192">
@@ -4866,7 +4836,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -4886,7 +4856,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194">
@@ -4906,7 +4876,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195">
@@ -4926,7 +4896,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="196">
@@ -4946,7 +4916,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="197">
@@ -4966,7 +4936,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="198">
@@ -4986,7 +4956,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="199">
@@ -5006,7 +4976,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="200">
@@ -5026,7 +4996,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -5046,7 +5016,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -5066,7 +5036,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203">
@@ -5086,7 +5056,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="204">
@@ -5106,7 +5076,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="205">
@@ -5126,7 +5096,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="206">
@@ -5146,7 +5116,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="207">
@@ -5166,7 +5136,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="208">
@@ -5186,7 +5156,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -5206,7 +5176,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -5226,7 +5196,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="211">
@@ -5246,7 +5216,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="212">
@@ -5266,7 +5236,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="213">
@@ -5286,7 +5256,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="214">
@@ -5306,7 +5276,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="215">
@@ -5326,7 +5296,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="216">
@@ -5346,7 +5316,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -5366,7 +5336,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218">
@@ -5386,7 +5356,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="219">
@@ -5406,7 +5376,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="220">
@@ -5426,7 +5396,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="221">
@@ -5446,7 +5416,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="222">
@@ -5466,7 +5436,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="223">
@@ -5486,7 +5456,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="224">
@@ -5506,7 +5476,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225">
@@ -5526,7 +5496,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226">
@@ -5546,7 +5516,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="227">
@@ -5566,7 +5536,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="228">
@@ -5586,7 +5556,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="229">
@@ -5606,7 +5576,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="230">
@@ -5626,7 +5596,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="231">
@@ -5646,7 +5616,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="232">
@@ -5666,7 +5636,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233">
@@ -5706,7 +5676,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="235">
@@ -5726,7 +5696,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="236">
@@ -5746,7 +5716,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="237">
@@ -5766,7 +5736,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="238">
@@ -5786,7 +5756,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="239">
@@ -5806,7 +5776,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="240">
@@ -5826,7 +5796,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="241">
@@ -5846,7 +5816,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="242">
@@ -5866,7 +5836,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="243">
@@ -5886,7 +5856,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="244">
@@ -5906,7 +5876,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="245">
@@ -5926,7 +5896,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="246">
@@ -5946,7 +5916,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="247">
@@ -5966,7 +5936,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="248">
@@ -5986,7 +5956,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="249">
@@ -6006,7 +5976,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="250">
@@ -6026,7 +5996,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="251">
@@ -6046,7 +6016,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="252">
@@ -6086,7 +6056,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="254">
@@ -6106,7 +6076,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="255">
@@ -6126,7 +6096,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="256">
@@ -6146,7 +6116,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257">
@@ -6166,7 +6136,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="258">
@@ -6186,7 +6156,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="259">
@@ -6206,7 +6176,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="260">
@@ -6226,7 +6196,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="261">
@@ -6246,7 +6216,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="262">
@@ -6266,7 +6236,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="263">
@@ -6326,7 +6296,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="266">
@@ -6386,7 +6356,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="269">
@@ -6406,7 +6376,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="270">
@@ -6426,7 +6396,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="271">
@@ -6446,7 +6416,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="272">
@@ -6466,7 +6436,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="273">
@@ -6506,7 +6476,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="275">
@@ -6526,7 +6496,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="276">
@@ -6546,7 +6516,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="277">
@@ -6566,7 +6536,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="278">
@@ -6586,7 +6556,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="279">
@@ -6606,7 +6576,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="280">
@@ -6646,7 +6616,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="282">
@@ -6666,7 +6636,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="283">
@@ -6686,7 +6656,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="284">
@@ -6706,7 +6676,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="285">
@@ -6726,7 +6696,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="286">
@@ -6746,7 +6716,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="287">
@@ -6766,7 +6736,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="288">
@@ -6786,7 +6756,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="289">
@@ -6806,7 +6776,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="290">
@@ -6826,7 +6796,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="291">
@@ -6846,7 +6816,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="292">
@@ -6866,7 +6836,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="293">
@@ -6886,7 +6856,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="294">
@@ -6906,7 +6876,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="295">
@@ -6926,7 +6896,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="296">
@@ -6946,7 +6916,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="297">
@@ -6966,7 +6936,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="298">
@@ -6986,7 +6956,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="299">
@@ -7006,7 +6976,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="300">
@@ -7026,7 +6996,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="301">
@@ -7046,7 +7016,7 @@
         </is>
       </c>
       <c r="D301" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="302">
@@ -7066,7 +7036,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="303">
@@ -7086,7 +7056,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="304">
@@ -7106,7 +7076,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
@@ -7126,7 +7096,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="306">
@@ -7146,7 +7116,7 @@
         </is>
       </c>
       <c r="D306" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="307">
@@ -7166,7 +7136,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="308">
@@ -7186,7 +7156,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="309">
@@ -7206,7 +7176,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="310">
@@ -7226,7 +7196,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="311">
@@ -7246,7 +7216,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="312">
@@ -7306,7 +7276,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="315">
@@ -7326,7 +7296,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="316">
@@ -7346,7 +7316,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="317">
@@ -7366,7 +7336,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="318">
@@ -7386,7 +7356,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="319">
@@ -7406,7 +7376,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="320">
@@ -7446,7 +7416,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="322">
@@ -7466,7 +7436,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="323">
@@ -7486,7 +7456,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="324">
@@ -7506,7 +7476,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="325">
@@ -7526,7 +7496,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="326">
@@ -7546,7 +7516,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="327">
@@ -7566,7 +7536,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="328">
@@ -7626,7 +7596,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="331">
@@ -7646,7 +7616,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="332">
@@ -7666,7 +7636,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="333">
@@ -7686,7 +7656,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="334">
@@ -7706,7 +7676,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="335">
@@ -7726,7 +7696,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="336">
@@ -7766,7 +7736,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="338">
@@ -7786,7 +7756,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="339">
@@ -7806,7 +7776,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="340">
@@ -7826,7 +7796,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="341">
@@ -7846,7 +7816,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="342">
@@ -7866,7 +7836,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="343">
@@ -7886,7 +7856,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="344">
@@ -7906,7 +7876,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="345">
@@ -7946,7 +7916,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="347">
@@ -7986,7 +7956,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="349">
@@ -8006,7 +7976,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="350">
@@ -8026,7 +7996,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="351">
@@ -8046,7 +8016,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="352">
@@ -8066,7 +8036,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
@@ -8086,7 +8056,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="354">
@@ -8106,7 +8076,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355">
@@ -8126,7 +8096,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="356">
@@ -8146,7 +8116,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="357">
@@ -8166,7 +8136,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="358">
@@ -8186,7 +8156,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="359">
@@ -8206,7 +8176,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360">
@@ -8296,7 +8266,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Supuesto de demostración: la farmacia abre todos los días. Cámbialo si no es así.</t>
+          <t>El sanatorio opera 24 horas todos los días (TuSalud y Facebook).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Costo por pedido S de Q35 a Q150: trabajo interno más flete
Q35 era solo lo que cobra una mensajería por una caja chica. El escenario
base ahora suma unos Q100 de trabajo interno (preparar, recibir, revisar y
registrar el pedido) y unos Q50 de flete al interior.

Cambia el valor por defecto, la ayuda de Configuración, la plantilla y el
ejemplo de importación (solo esa celda) y la documentación. La tabla de
resultados de la simulación se recalculó con Q150 (80 días, mismas
semillas): SALVAMED pasa a 10-12 envíos y gasta entre 35 % y 43 % de lo
del Roble hoy.

La base de producción guarda su propio valor: hay que cambiarlo en
Configuración → Costo por pedido.
</commit_message>
<xml_diff>
--- a/datos/ejemplo_simulado.xlsx
+++ b/datos/ejemplo_simulado.xlsx
@@ -8307,11 +8307,11 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>35</v>
+        <v>150</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>S en quetzales. Escenario base: solo el envío.</t>
+          <t>S en quetzales. Escenario base: unos Q100 de trabajo interno y unos Q50 de flete.</t>
         </is>
       </c>
     </row>

</xml_diff>